<commit_message>
feat(F-NAR-019): ATOM-DIF.PAR.002-06 Mila laisse le temps à Victorino
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.002-06.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.002-06.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le papillon de papier</t>
+          <t>Mila laisse le temps à Victorino</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>salon, canapé, papillon de papier, ailes jaunes, rideau, linge séché, fenêtre</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nina, Nino, maman</t>
+          <t>Mila, Victorino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Un papillon de papier attend sur la table. Nino veut raconter. Nina connaît le mot. Elle attend. Il dit papillon, puis les ailes jaunes.</t>
+          <t>Une aile jaune tremble sur le canapé. Sur le tissu, un éclat de canapé brille. Mila veut le faire voler, maintenant. Victorino dit : j'ai vu. Le mot coincé. Elle connaît, ouvre la bouche maintenant, Papillon trop tôt. Sourire parti, papa accroupi. Elle referme, attend. Merci vécu. 2e ruse, Dis-le, ailes jaunes. Un éclat de canapé tient sur le tissu.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un rayon traverse le salon tout entier. Dedans, la poussière danse tout doucement. Le rideau bouge, à peine. Ça sent le linge propre. Je plie les serviettes, Nina. Elles sont encore un peu chaudes. Je peux aider ? Oui. Une petite pile, là. En ce moment, Nina est près de la table. Le bois de la table est lisse et tiède. Tu poses la pile ici, tout droit. Elle est chaude, la serviette. Oui. Ça sent le propre. Un papillon de papier est posé dessus. Ses ailes sont jaunes, un peu froissées. Nino arrive avec ses chaussettes silencieuses. J'ai vu... Il s'arrête. Il cherche le mot. Nina connaît le mot. Elle ouvre la bouche. On peut laisser le temps, Nina. On attend la fin de la phrase. Nina referme la bouche. Elle pose une serviette bien à plat. Elle attend. Le rideau bouge encore. J'ai vu un papillon. Il est en papier. Oui. Papier. Bravo, Nina. Tu as su attendre. Nino touche une aile, tout doux. Les ailes sont... Nina attend encore. Un grain de poussière passe dans le rayon. Les ailes sont jaunes. Jaunes, oui. Vous parlez l'un après l'autre. Nina, tu as laissé le temps ? Oui, maman. On écoute jusqu'au bout. Maman pose deux coussins. On s'assoit ? Moi, je... Nino cherche encore un mot. Nina attend la fin. Moi, je veux le coussin bleu. D'accord. Le bleu. Ils s'assoient. Le papillon reste sur la table. Nina a su laisser le temps. On plie encore une serviette ? Oui. Elle est tiède. Nino attend, les mains sur le coussin. Le rayon touche une aile jaune.</t>
+          <t>Le soleil pose une bande chaude sur le canapé. Le tissu sent le linge séché. Il est chaud, papa. Tu le sens, le canapé ? Oui, papa. Une aile de papier tremble, jaune. Elle bouge, maman. Le papillon est en papier, Mila ? Oui, maman. Sur le tissu, un éclat de canapé brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Le rideau laisse passer l'air. Ça sent le propre. Le linge a séché, Mila ? Oui, maman. Le papillon de papier attend sur le bras. Le papier est lisse, contre la paume. Il est lisse, maman. Tu le tiens, Mila ? Oui. En ce moment, Mila pose le papillon. Je veux le faire voler, maintenant ! Jusqu'à la fenêtre, tout de suite. Le papillon jaune, là ? Oui, le jaune. Les ailes sont un peu froissées ? Un peu. Victorino arrive près du canapé. Il marche sans bruit. Tu l'as vu, toi ? Victorino ouvre la bouche. J'ai vu. Il s'arrête. Le mot reste coincé. Mila connaît le mot. Le mot monte très vite. Elle ouvre la bouche, maintenant. Papillon ! Le mot sort trop tôt. Victorino recule un peu. Il serre les lèvres. Oh. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Victorino, Mila ? Oui, papa. Tes lèvres sont ouvertes, Mila ? Un peu, maman. L'éclat de canapé tremble, puis tient. Victorino reste près du bras. Le mot manque, papa. Mila regarde papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un rayon traverse le salon tout entier. Dedans, la poussière danse tout doucement. Le rideau bouge, à peine. Ça sent le linge propre. Je plie les serviettes, Nina. Elles sont encore un peu chaudes. Je peux aider ? Oui. Une petite pile, là. En ce moment, Nina est près de la table. Le bois de la table est lisse et tiède. Tu poses la pile ici, tout droit. Elle est chaude, la serviette. Oui. Ça sent le propre. Un papillon de papier est posé dessus. Ses ailes sont jaunes, un peu froissées. Nino arrive avec ses chaussettes silencieuses. J'ai vu... Il s'arrête. Il cherche le mot. Nina connaît le mot. Elle ouvre la bouche. On peut laisser le temps, Nina. On attend la fin de la phrase. Nina referme la bouche. Elle pose une serviette bien à plat. Elle attend. Le rideau bouge encore. J'ai vu un papillon. Il est en papier. Oui. Papier. Bravo, Nina. Tu as su attendre. Nino touche une aile, tout doux. Les ailes sont... Nina attend encore. Un grain de poussière passe dans le rayon. Les ailes sont jaunes. Jaunes, oui. Vous parlez l'un après l'autre. Nina, tu as laissé le temps ? Oui, maman. On écoute jusqu'au bout. Maman pose deux coussins. On s'assoit ? Moi, je... Nino cherche encore un mot. Nina attend la fin. Moi, je veux le coussin bleu. D'accord. Le bleu. Ils s'assoient. Le papillon reste sur la table. Nina a su laisser le temps. On plie encore une serviette ? Oui. Elle est tiède. Nino attend, les mains sur le coussin. Le rayon touche une aile jaune.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soleil pose une bande chaude sur le canapé. Le tissu sent le linge séché. Il est chaud, papa. Tu le sens, le canapé ? Oui, papa. Une aile de papier tremble, jaune. Elle bouge, maman. Le papillon est en papier, Mila ? Oui, maman. Sur le tissu, un &lt;emphasis level="moderate"&gt;éclat de canapé&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Le rideau laisse passer l'air. Ça sent le propre. Le linge a séché, Mila ? Oui, maman. Le papillon de papier attend sur le bras. Le papier est lisse, contre la paume. Il est lisse, maman. Tu le tiens, Mila ? Oui. En ce moment, Mila pose le papillon. Je veux le faire voler, maintenant ! Jusqu'à la fenêtre, tout de suite. Le papillon jaune, là ? Oui, le jaune. Les ailes sont un peu froissées ? Un peu. Victorino arrive près du canapé. Il marche sans bruit. Tu l'as vu, toi ? Victorino ouvre la bouche. J'ai vu. Il s'arrête. Le mot reste coincé. Mila connaît le mot. Le mot monte très vite. Elle ouvre la bouche, maintenant. Papillon ! Le mot sort trop tôt. Victorino recule un peu. Il serre les lèvres. Oh. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Victorino, Mila ? Oui, papa. Tes lèvres sont ouvertes, Mila ? Un peu, maman. L'éclat de canapé tremble, puis tient. Victorino reste près du bras. Le mot manque, papa. Mila regarde papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Hortense est dans le salon avec maman. Eliott veut raconter. Il dit : j'ai vu.. Puis il cherche le mot. Hortense connaît le mot. Elle ouvre la bouche. Maman dit : on peut &lt;emphasis&gt;laisser&lt;/emphasis&gt; le temps. On n'achève pas à sa place. Hortense attend la fin de la phrase. Eliott dit : j'ai vu un papillon. Hortense sourit. Elle a su laisser le temps. [pause]</t>
+          <t>Le soleil pose une bande chaude sur le canapé. Le tissu sent le linge séché. Il est chaud, papa. Tu le sens, le canapé ? Oui, papa. Une aile de papier tremble, jaune. Elle bouge, maman. Le papillon est en papier, Mila ? Oui, maman. Sur le tissu, un &lt;emphasis&gt;éclat de canapé&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Le rideau laisse passer l'air. Ça sent le propre. Le linge a séché, Mila ? Oui, maman. Le papillon de papier attend sur le bras. Le papier est lisse, contre la paume. Il est lisse, maman. Tu le tiens, Mila ? Oui. En ce moment, Mila pose le papillon. Je veux le faire voler, maintenant ! Jusqu'à la fenêtre, tout de suite. Le papillon jaune, là ? Oui, le jaune. Les ailes sont un peu froissées ? Un peu. Victorino arrive près du canapé. Il marche sans bruit. Tu l'as vu, toi ? Victorino ouvre la bouche. J'ai vu. Il s'arrête. Le mot reste coincé. Mila connaît le mot. Le mot monte très vite. Elle ouvre la bouche, maintenant. Papillon ! Le mot sort trop tôt. Victorino recule un peu. Il serre les lèvres. Oh. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Victorino, Mila ? Oui, papa. Tes lèvres sont ouvertes, Mila ? Un peu, maman. L'éclat de canapé tremble, puis tient. Victorino reste près du bras. Le mot manque, papa. Mila regarde papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>laisser</t>
+          <t>éclat de canapé</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,70 +1321,74 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_voler_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un rayon traverse le salon tout entier.
-narrateur|Dedans, la poussière danse tout doucement.
-narrateur|Le rideau bouge, à peine.
-narrateur|Ça sent le linge propre.
-maman|Je plie les serviettes, Nina.
-maman|Elles sont encore un peu chaudes.
-enfant-f|Je peux aider ?
-maman|Oui.
-maman|Une petite pile, là.
-narrateur|En ce moment, Nina est près de la table.
-narrateur|Le bois de la table est lisse et tiède.
-maman|Tu poses la pile ici, tout droit.
-enfant-f|Elle est chaude, la serviette.
-maman|Oui.
-maman|Ça sent le propre.
-narrateur|Un papillon de papier est posé dessus.
-narrateur|Ses ailes sont jaunes, un peu froissées.
-narrateur|Nino arrive avec ses chaussettes silencieuses.
-copain|J'ai vu...
+          <t>narrateur|Le soleil pose une bande chaude sur le canapé.
+narrateur|Le tissu sent le linge séché.
+enfant-f|Il est chaud, papa.
+papa|Tu le sens, le canapé ?
+enfant-f|Oui, papa.
+narrateur|Une aile de papier tremble, jaune.
+enfant-f|Elle bouge, maman.
+maman|Le papillon est en papier, Mila ?
+enfant-f|Oui, maman.
+narrateur|Sur le tissu, un éclat de canapé brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Le rideau laisse passer l'air.
+enfant-f|Ça sent le propre.
+maman|Le linge a séché, Mila ?
+enfant-f|Oui, maman.
+narrateur|Le papillon de papier attend sur le bras.
+narrateur|Le papier est lisse, contre la paume.
+enfant-f|Il est lisse, maman.
+maman|Tu le tiens, Mila ?
+enfant-f|Oui.
+narrateur|En ce moment, Mila pose le papillon.
+enfant-f|Je veux le faire voler, maintenant !
+enfant-f|Jusqu'à la fenêtre, tout de suite.
+papa|Le papillon jaune, là ?
+enfant-f|Oui, le jaune.
+maman|Les ailes sont un peu froissées ?
+enfant-f|Un peu.
+narrateur|Victorino arrive près du canapé.
+narrateur|Il marche sans bruit.
+enfant-f|Tu l'as vu, toi ?
+narrateur|Victorino ouvre la bouche.
+copain|J'ai vu.
 narrateur|Il s'arrête.
-narrateur|Il cherche le mot.
-narrateur|Nina connaît le mot.
-narrateur|Elle ouvre la bouche.
-maman|On peut laisser le temps, Nina.
-maman|On attend la fin de la phrase.
-narrateur|Nina referme la bouche.
-narrateur|Elle pose une serviette bien à plat.
-narrateur|Elle attend.
-narrateur|Le rideau bouge encore.
-copain|J'ai vu un papillon.
-enfant-f|Il est en papier.
-copain|Oui.
-copain|Papier.
-maman|Bravo, Nina.
-maman|Tu as su attendre.
-narrateur|Nino touche une aile, tout doux.
-copain|Les ailes sont...
-narrateur|Nina attend encore.
-narrateur|Un grain de poussière passe dans le rayon.
-copain|Les ailes sont jaunes.
-enfant-f|Jaunes, oui.
-maman|Vous parlez l'un après l'autre.
-maman|Nina, tu as laissé le temps ?
-enfant-f|Oui, maman.
-maman|On écoute jusqu'au bout.
-narrateur|Maman pose deux coussins.
-maman|On s'assoit ?
-copain|Moi, je...
-narrateur|Nino cherche encore un mot.
-narrateur|Nina attend la fin.
-copain|Moi, je veux le coussin bleu.
-enfant-f|D'accord.
-enfant-f|Le bleu.
-narrateur|Ils s'assoient.
-narrateur|Le papillon reste sur la table.
-narrateur|Nina a su laisser le temps.
-maman|On plie encore une serviette ?
-enfant-f|Oui.
-enfant-f|Elle est tiède.
-narrateur|Nino attend, les mains sur le coussin.
-narrateur|Le rayon touche une aile jaune.</t>
+narrateur|Le mot reste coincé.
+narrateur|Mila connaît le mot.
+narrateur|Le mot monte très vite.
+narrateur|Elle ouvre la bouche, maintenant.
+enfant-f|Papillon !
+narrateur|Le mot sort trop tôt.
+narrateur|Victorino recule un peu.
+narrateur|Il serre les lèvres.
+enfant-f|Oh.
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Victorino, Mila ?
+enfant-f|Oui, papa.
+maman|Tes lèvres sont ouvertes, Mila ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de canapé tremble, puis tient.
+narrateur|Victorino reste près du bras.
+enfant-f|Le mot manque, papa.
+narrateur|Mila regarde papa.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>salon,papier</t>
         </is>
       </c>
     </row>
@@ -1411,17 +1415,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Nino cherche un mot. Que fait Nina ?</t>
+          <t>Victorino cherche un mot. Que fait Mila ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nino cherche un mot. Que fait Nina ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorino cherche un mot. Que fait &lt;emphasis level="moderate"&gt;Mila&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Eliott cherche un mot. Que fait Hortense ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorino cherche un mot. Que fait &lt;emphasis&gt;Mila&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1484,7 +1488,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1495,7 +1499,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1510,34 +1514,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Mila</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1552,23 +1560,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=victorino_cherche_un_mot_que_fait_mila; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Nino cherche un mot.
-narrateur|Que fait Nina ?</t>
+          <t>narrateur|Victorino cherche un mot.
+narrateur|Que fait Mila ?</t>
         </is>
       </c>
     </row>
@@ -1595,17 +1603,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina a su laisser le temps. Nino a fini sa phrase. On attend la fin de la phrase. Bravo, Nina. J'ai laissé le temps.</t>
+          <t>Mila veut le mot, tout de suite. Papillon, maintenant ! Elle ouvre la bouche. Les mots se bousculent dans sa bouche. Victorino recule un peu. Il serre les mains contre lui. Oh. Le sourire ne revient pas. Mila referme la bouche. Personne ne parle. Elle observe le papillon, un instant. Elle écoute le rideau, tout près. Tu veux voler avec Victorino ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le papillon, puis on reste. D'accord. Mila reste un moment, les lèvres fermées. Elle attend. J'ai vu un papillon. Il est en papier. Oui. Papier. Merci, Mila. Papa a vu les deux, au salon. Le papier est lisse, sous les doigts. Il est lisse. Une aile jaune repose sur le bras. Le papillon. Il a des ailes, là ? Oui, là. Mila glisse la main sur le tissu. Le canapé est doux, contre la peau. Tes mains sont au chaud, Mila ? Un peu, maman. Victorino s'assoit, puis se relève. Papillon. On va jusqu'à la fenêtre ? La fenêtre est près du rideau. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina a su laisser le temps. Nino a fini sa phrase. On attend la fin de la phrase. Bravo, Nina. J'ai laissé le temps.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila veut le mot, tout de suite. Papillon, maintenant ! Elle ouvre la bouche. Les mots se bousculent dans sa bouche. Victorino recule un peu. Il serre les mains contre lui. Oh. Le sourire ne revient pas. Mila referme la bouche. Personne ne parle. Elle observe le &lt;emphasis level="moderate"&gt;papillon&lt;/emphasis&gt;, un instant. Elle écoute le rideau, tout près. Tu veux voler avec Victorino ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le papillon, puis on reste. D'accord. Mila reste un moment, les lèvres fermées. Elle attend. J'ai vu un papillon. Il est en papier. Oui. Papier. Merci, Mila. Papa a vu les deux, au salon. Le papier est lisse, sous les doigts. Il est lisse. Une aile jaune repose sur le bras. Le papillon. Il a des ailes, là ? Oui, là. Mila glisse la main sur le tissu. Le canapé est doux, contre la peau. Tes mains sont au chaud, Mila ? Un peu, maman. Victorino s'assoit, puis se relève. Papillon. On va jusqu'à la fenêtre ? La fenêtre est près du rideau. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Hortense a su &lt;emphasis&gt;laisser&lt;/emphasis&gt; le temps. Eliott a fini sa phrase. [pause]</t>
+          <t>Mila veut le mot, tout de suite. Papillon, maintenant ! Elle ouvre la bouche. Les mots se bousculent dans sa bouche. Victorino recule un peu. Il serre les mains contre lui. Oh. Le sourire ne revient pas. Mila referme la bouche. Personne ne parle. Elle observe le &lt;emphasis&gt;papillon&lt;/emphasis&gt;, un instant. Elle écoute le rideau, tout près. Tu veux voler avec Victorino ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le papillon, puis on reste. D'accord. Mila reste un moment, les lèvres fermées. Elle attend. J'ai vu un papillon. Il est en papier. Oui. Papier. Merci, Mila. Papa a vu les deux, au salon. Le papier est lisse, sous les doigts. Il est lisse. Une aile jaune repose sur le bras. Le papillon. Il a des ailes, là ? Oui, là. Mila glisse la main sur le tissu. Le canapé est doux, contre la peau. Tes mains sont au chaud, Mila ? Un peu, maman. Victorino s'assoit, puis se relève. Papillon. On va jusqu'à la fenêtre ? La fenêtre est près du rideau. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1652,7 +1660,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1660,10 +1668,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1686,30 +1694,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>laisser</t>
+          <t>papillon</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1718,10 +1726,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1734,16 +1742,56 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_ouvre_referme_attend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina a su laisser le temps.
-narrateur|Nino a fini sa phrase.
-maman|On attend la fin de la phrase.
-maman|Bravo, Nina.
-enfant-f|J'ai laissé le temps.</t>
+          <t>narrateur|Mila veut le mot, tout de suite.
+enfant-f|Papillon, maintenant !
+narrateur|Elle ouvre la bouche.
+narrateur|Les mots se bousculent dans sa bouche.
+narrateur|Victorino recule un peu.
+narrateur|Il serre les mains contre lui.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Mila referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe le papillon, un instant.
+narrateur|Elle écoute le rideau, tout près.
+papa|Tu veux voler avec Victorino ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Papa, on fait quoi ?
+papa|On pose le papillon, puis on reste.
+enfant-f|D'accord.
+narrateur|Mila reste un moment, les lèvres fermées.
+narrateur|Elle attend.
+copain|J'ai vu un papillon.
+enfant-f|Il est en papier.
+copain|Oui.
+copain|Papier.
+papa|Merci, Mila.
+narrateur|Papa a vu les deux, au salon.
+maman|Le papier est lisse, sous les doigts.
+enfant-f|Il est lisse.
+narrateur|Une aile jaune repose sur le bras.
+enfant-f|Le papillon.
+papa|Il a des ailes, là ?
+enfant-f|Oui, là.
+narrateur|Mila glisse la main sur le tissu.
+narrateur|Le canapé est doux, contre la peau.
+maman|Tes mains sont au chaud, Mila ?
+enfant-f|Un peu, maman.
+narrateur|Victorino s'assoit, puis se relève.
+copain|Papillon.
+enfant-f|On va jusqu'à la fenêtre ?
+maman|La fenêtre est près du rideau.
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>salon,papier</t>
         </is>
       </c>
     </row>
@@ -1770,17 +1818,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman pose encore un coussin. Vous êtes bien assis ? Oui, maman. Le papillon reste là. Oui. On le regarde ensemble. Il veut... Nina attend la fin. Il veut voler. Il reste sur la table. Tu as laissé le temps, Nina. Le rayon a un peu bougé. La poussière danse encore.</t>
+          <t>Ils restent près du canapé. Le papillon jaune penche vers le bras. Je le fais voler, maintenant ! Mila pousse trop vite. L'aile glisse sur le tissu. Ça glisse ! Dis-le, Victorino ! Victorino serre les lèvres. Mila avance les mots, trop vite. Puis elle s'arrête net. Mila referme la bouche, cette fois. Ses lèvres se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le papillon, un instant. Elle écoute le rideau, tout près. Près du bras, un éclat de canapé luit. Là, sur le canapé. Tu prends le papillon, Victorino ? Victorino ne dit rien. Il tend les mains, sans parler. Les ailes sont. Mila attend. Les ailes sont jaunes. Jaunes, oui. Mila passe le papillon, sans se presser. Victorino le reçoit, plus lentement. Le papier est lisse et tiède. Tu le vois, le papillon ? Oui, papa. L'aile est tiède, Mila ? Oui, maman. Victorino souffle, un filet d'air. L'aile se lève un peu, puis retombe. L'aile bouge, Mila ? Oui, papa. Il veut. Mila attend. Il veut voler. Il vole un peu. Un rayon passe sur le canapé. Il allume le tissu.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman pose encore un coussin. Vous êtes bien assis ? Oui, maman. Le papillon reste là. Oui. On le regarde ensemble. Il veut... Nina attend la fin. Il veut voler. Il reste sur la table. Tu as laissé le temps, Nina. Le rayon a un peu bougé. La poussière danse encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent près du canapé. Le papillon jaune penche vers le bras. Je le fais voler, maintenant ! Mila pousse trop vite. L'aile glisse sur le tissu. Ça glisse ! Dis-le, Victorino ! Victorino serre les lèvres. Mila avance les mots, trop vite. Puis elle s'arrête net. Mila referme la bouche, cette fois. Ses lèvres se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le papillon, un instant. Elle écoute le rideau, tout près. Près du bras, un &lt;emphasis level="moderate"&gt;éclat de canapé&lt;/emphasis&gt; luit. Là, sur le canapé. Tu prends le papillon, Victorino ? Victorino ne dit rien. Il tend les mains, sans parler. Les ailes sont. Mila attend. Les ailes sont jaunes. Jaunes, oui. Mila passe le papillon, sans se presser. Victorino le reçoit, plus lentement. Le papier est lisse et tiède. Tu le vois, le papillon ? Oui, papa. L'aile est tiède, Mila ? Oui, maman. Victorino souffle, un filet d'air. L'aile se lève un peu, puis retombe. L'aile bouge, Mila ? Oui, papa. Il veut. Mila attend. Il veut voler. Il vole un peu. Un rayon passe sur le canapé. Il allume le tissu.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman pose deux coussins. Ils s'assoient. [pause]</t>
+          <t>Ils restent près du canapé. Le papillon jaune penche vers le bras. Je le fais voler, maintenant ! Mila pousse trop vite. L'aile glisse sur le tissu. Ça glisse ! Dis-le, Victorino ! Victorino serre les lèvres. Mila avance les mots, trop vite. Puis elle s'arrête net. Mila referme la bouche, cette fois. Ses lèvres se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le papillon, un instant. Elle écoute le rideau, tout près. Près du bras, un &lt;emphasis&gt;éclat de canapé&lt;/emphasis&gt; luit. Là, sur le canapé. Tu prends le papillon, Victorino ? Victorino ne dit rien. Il tend les mains, sans parler. Les ailes sont. Mila attend. Les ailes sont jaunes. Jaunes, oui. Mila passe le papillon, sans se presser. Victorino le reçoit, plus lentement. Le papier est lisse et tiède. Tu le vois, le papillon ? Oui, papa. L'aile est tiède, Mila ? Oui, maman. Victorino souffle, un filet d'air. L'aile se lève un peu, puis retombe. L'aile bouge, Mila ? Oui, papa. Il veut. Mila attend. Il veut voler. Il vole un peu. Un rayon passe sur le canapé. Il allume le tissu. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1827,7 +1875,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1835,10 +1883,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1859,28 +1907,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de canapé</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1889,10 +1941,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1903,22 +1955,59 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=dis_le_ailes_jaunes_elle_referme; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman pose encore un coussin.
-maman|Vous êtes bien assis ?
+          <t>narrateur|Ils restent près du canapé.
+narrateur|Le papillon jaune penche vers le bras.
+enfant-f|Je le fais voler, maintenant !
+narrateur|Mila pousse trop vite.
+narrateur|L'aile glisse sur le tissu.
+enfant-f|Ça glisse !
+enfant-f|Dis-le, Victorino !
+narrateur|Victorino serre les lèvres.
+narrateur|Mila avance les mots, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Mila referme la bouche, cette fois.
+narrateur|Ses lèvres se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le papillon, un instant.
+narrateur|Elle écoute le rideau, tout près.
+narrateur|Près du bras, un éclat de canapé luit.
+enfant-f|Là, sur le canapé.
+enfant-f|Tu prends le papillon, Victorino ?
+narrateur|Victorino ne dit rien.
+narrateur|Il tend les mains, sans parler.
+copain|Les ailes sont.
+narrateur|Mila attend.
+copain|Les ailes sont jaunes.
+enfant-f|Jaunes, oui.
+narrateur|Mila passe le papillon, sans se presser.
+narrateur|Victorino le reçoit, plus lentement.
+narrateur|Le papier est lisse et tiède.
+papa|Tu le vois, le papillon ?
+enfant-f|Oui, papa.
+maman|L'aile est tiède, Mila ?
 enfant-f|Oui, maman.
-copain|Le papillon reste là.
-maman|Oui.
-maman|On le regarde ensemble.
-copain|Il veut...
-narrateur|Nina attend la fin.
+narrateur|Victorino souffle, un filet d'air.
+narrateur|L'aile se lève un peu, puis retombe.
+papa|L'aile bouge, Mila ?
+enfant-f|Oui, papa.
+copain|Il veut.
+narrateur|Mila attend.
 copain|Il veut voler.
-enfant-f|Il reste sur la table.
-maman|Tu as laissé le temps, Nina.
-narrateur|Le rayon a un peu bougé.
-narrateur|La poussière danse encore.</t>
+enfant-f|Il vole un peu.
+maman|Un rayon passe sur le canapé.
+enfant-f|Il allume le tissu.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>salon,papier</t>
         </is>
       </c>
     </row>
@@ -1945,17 +2034,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai attendu la fin. Bravo. Les ailes jaunes restent ouvertes.</t>
+          <t>Ils restent près du canapé. Le papillon est là, Mila ? Oui, maman. Tu souffles un peu ? Oui, papa. Mila souffle, un filet d'air. Le papier sent bon. Tu le sens, le papillon ? Oui, maman. Le tissu reste un peu, chaud. Il a tenu, sous l'aile. Papillon. Le papillon jaune fait de l'ombre. Le rideau s'éloigne, sans bruit. On le fait voler, après. Un éclat de canapé tient sur le tissu.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai attendu la fin. Bravo. Les ailes jaunes restent ouvertes.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du canapé. Le papillon est là, Mila ? Oui, maman. Tu souffles un peu ? Oui, papa. Mila souffle, un filet d'air. Le papier sent bon. Tu le sens, le papillon ? Oui, maman. Le tissu reste un peu, chaud. Il a tenu, sous l'aile. Papillon. Le papillon jaune fait de l'ombre. Le rideau s'éloigne, sans bruit. On le fait voler, après. Un &lt;emphasis level="moderate"&gt;éclat de canapé&lt;/emphasis&gt; tient sur le tissu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du canapé. Le papillon est là, Mila ? Oui, maman. Tu souffles un peu ? Oui, papa. Mila souffle, un filet d'air. Le papier sent bon. Tu le sens, le papillon ? Oui, maman. Le tissu reste un peu, chaud. Il a tenu, sous l'aile. Papillon. Le papillon jaune fait de l'ombre. Le rideau s'éloigne, sans bruit. On le fait voler, après. Un &lt;emphasis&gt;éclat de canapé&lt;/emphasis&gt; tient sur le tissu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2002,7 +2091,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2010,10 +2099,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2022,12 +2111,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2036,17 +2125,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de canapé</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2055,11 +2148,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2068,26 +2161,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_tissu; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai attendu la fin.
-maman|Bravo.
-narrateur|Les ailes jaunes restent ouvertes.</t>
+          <t>narrateur|Ils restent près du canapé.
+maman|Le papillon est là, Mila ?
+enfant-f|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-f|Oui, papa.
+narrateur|Mila souffle, un filet d'air.
+enfant-f|Le papier sent bon.
+maman|Tu le sens, le papillon ?
+enfant-f|Oui, maman.
+papa|Le tissu reste un peu, chaud.
+enfant-f|Il a tenu, sous l'aile.
+copain|Papillon.
+narrateur|Le papillon jaune fait de l'ombre.
+narrateur|Le rideau s'éloigne, sans bruit.
+enfant-f|On le fait voler, après.
+narrateur|Un éclat de canapé tient sur le tissu.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>salon,canapé</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2172,6 +2287,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>